<commit_message>
Add proposed 'Missing Coverage' sheet to the QA workbook
33 test cases identified as gaps in the original 164-case suite (6
security, 25 functional across every pipeline stage, 2 performance),
added as a new sheet in both the original spreadsheet and the executed
copy. Not tested/executed -- Actual Result left blank, Status "Not Run"
for all of them, per instruction to identify gaps without running them.

Security-relevant gaps (CSV/formula injection, SSRF via scraped URLs,
ReDoS on the LLM-generated phone_regex, API key enforcement) were
grounded by reading the actual code paths, not assumed.
</commit_message>
<xml_diff>
--- a/qa/professional_qa/AI_BDM_Professional_QA_Test_Cases_EXECUTED.xlsx
+++ b/qa/professional_qa/AI_BDM_Professional_QA_Test_Cases_EXECUTED.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Coverage Matrix" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Defect Log" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Missing Coverage (Proposed)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$N$165</definedName>
@@ -36,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +59,12 @@
         <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -76,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,6 +106,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -11182,4 +11190,2086 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Test Data / Input</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>Defect ID</t>
+        </is>
+      </c>
+      <c r="N1" s="8" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GAP-SEC-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CSV/formula injection</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Malicious field value scraped from a business website</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Run storage export</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A scraped business name/field begins with '=', '+', '-', or '@' (e.g. '=cmd|...')</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Discover/qualify a business whose scraped name or field starts with a formula-trigger character; export crawl_index.csv; open in Excel/Sheets.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Exported CSV never lets a field value execute as a formula when opened in a spreadsheet application (leading formula-trigger characters are neutralized/escaped).</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GAP-SEC-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SSRF via discovered/scraped URLs</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Search result or on-page link points at an internal/private address</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Run discovery/scraping</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A malicious page links to http://169.254.169.254/ (cloud metadata) or a localhost/private-range address</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Have discovery or the internal-link crawler encounter such a URL and attempt to fetch it.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>The fetch layer refuses to request private/internal/link-local IP ranges; the business is skipped or the offending URL is dropped, not fetched.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GAP-SEC-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ReDoS via LLM-generated phone_regex</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Planner-generated phone_regex is adversarially pathological</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Run query planning + contact extraction</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>A phone_regex value with catastrophic-backtracking potential despite being short (e.g. "(a+)+$")</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Force or simulate the planner returning such a regex, then run contact extraction against a long block of scraped text.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Regex execution completes in bounded time (or the compiled regex is rejected/timed out) -- extraction never hangs the pipeline. The existing MAX_PHONE_REGEX_LEN length cap alone is not sufficient evidence; this must be probed directly.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GAP-SEC-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>API key auth enforcement</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Request made to a protected endpoint</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>API running</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>POST /api/v1/pipeline/run with (a) no X-API-Key header, (b) an invalid key</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Send both requests and inspect the response.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Both requests are rejected with 401/403 before any pipeline work starts; no research is executed and no leads are consumed.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GAP-SEC-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Denial-of-wallet / run cost ceiling</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Adversarial or runaway query</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Submit a query designed to maximize LLM/API calls (e.g. deliberately ambiguous, triggering many query-variation rounds)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A single query or a burst of concurrent job submissions</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Observe total LLM/API spend for one run and for a burst of submissions.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>A per-run or per-tenant cost/call ceiling exists and is enforced; a single adversarial query cannot cause unbounded spend.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GAP-SEC-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tenant isolation</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Two distinct tenant_ref values</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Submit jobs as two different tenants</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>tenant_ref='tenant-a' and tenant_ref='tenant-b' with overlapping queries</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Submit jobs for both tenants and inspect job listing/results/storage access.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tenant A can never list, read, or cancel Tenant B's jobs or results -- tenant_ref is enforced as an isolation boundary, not just a label.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Query Planning</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Non-English query text</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Application running</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>"Islamabad mein 3 dental clinics dhoondo" (Roman Urdu) or a fully non-Latin-script query</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Submit query and inspect generated plan.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Plan correctly extracts industry/location/count, or needs_clarification is set honestly if the model cannot parse it -- never a silently wrong/empty plan.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Query Planning</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Extremely long query</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Application running</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>A query several thousand characters long (e.g. pasted document text)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Submit query and inspect generated plan / any truncation behavior.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Query is handled without crashing or truncating in a way that silently drops the actual request; a graceful length-limit response is acceptable.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-003</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Query Planning</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Total planner failure</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Both primary and fallback planning models fail</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Simulate/force both LLM tiers to error or exhaust retries</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Submit a normal query while both models are unavailable.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>A clear, honest error/needs_clarification response is returned -- never a fabricated plan or a crash.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-004</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Query Planning</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Conflicting multi-location query</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Application running</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>"find 3 dentists in Islamabad or Lahore"</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Submit query and inspect generated plan.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Plan either clarifies the ambiguity or picks a defensible interpretation (e.g. treats as two valid locations) -- never silently drops one location without any signal.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Discovery &amp; Scraping</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Redirect loop</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>A discovered site redirects to itself or in a cycle</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>A target URL that HTTP-redirects in a loop</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Attempt to scrape the site.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>The fetch is bounded by a redirect-count limit and fails gracefully -- no hang.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-006</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Discovery &amp; Scraping</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Non-HTML content at a page URL</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>A discovered link resolves to a PDF/image, not HTML</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>A business page link that serves a PDF or image content-type</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Attempt to scrape/extract text from it.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>The page is skipped or handled as empty content, never crashes text extraction.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-007</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Discovery &amp; Scraping</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Premium scraper (ScrapingBee) quota/rate-limit failure</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ScrapingBee account exhausted/rate-limited</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>A site that requires premium scraping (native fetch blocked)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Attempt scraping when ScrapingBee itself errors.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Pipeline degrades gracefully (skips or native-fetch-falls-back) without crashing -- same class of guarantee already proven for the Serper-quota case.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-008</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Discovery &amp; Scraping</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Business with no website, Maps-only</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>A real business exists only as a Maps/directory listing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>A query targeting a category with some website-less businesses</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Run discovery + Maps enrichment.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>The business is still captured via the Maps stage and not silently dropped just because Stage 2 found no website to scrape.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-009</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Route Planner</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Single-page site</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>A business site has only one page (the homepage)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>A minimal one-page site</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Run route selection.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Route planner selects the single available page without error; no off-by-one/empty-list failure.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-010</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Route Planner</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Zero-useful-page site</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Every crawled page is filtered as noise</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>A site whose only pages are /cart, /wishlist, /privacy etc.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Run route selection.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Route planner returns an empty/near-empty selection and the pipeline reports this honestly downstream rather than erroring.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-011</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Route Planner</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tied retrieval scores</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Two or more pages score identically</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pages with equal BM25/embedding scores</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Run route selection twice on the same input.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Selection is deterministic across repeated runs (stable tie-breaking), not order-dependent randomness.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-012</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Stage 4</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Final Reasoning</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Contradictory evidence across pages</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Two pages of the same business disagree</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>e.g. one page says 'no online booking', another page's footer widget says 'book now'</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Run reasoning over both pages as evidence.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>The answer either reflects the more authoritative/recent signal or flags the contradiction -- never silently picks one at random without justification in the reasoning trace.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-013</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Stage 4</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Final Reasoning</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Evidence exceeding context window</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Route planner selects many/large pages</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>8 large selected pages whose combined text is very large</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Run reasoning with maximal evidence volume.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Evidence is truncated/summarized safely without an API error or a context-length crash.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-014</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Stage 5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Technology Detection</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Site behind bot-challenge (WAF/Cloudflare)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Detection fetch is blocked by a challenge page</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>A site returning a Cloudflare/WAF challenge page instead of real content</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Run detection against it.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Detection reports low-confidence/unknown rather than misreporting the challenge page's own tech signature as the business's tech stack.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-015</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Stage 6</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Chroma collection reuse across process restarts</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Same domain queried in two separate process runs</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Same business queried twice in separate Python process invocations</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Compare ingestion/query behavior across the restart.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Behavior is documented and consistent -- either the collection is correctly reused (no duplicate re-ingestion) or correctly rebuilt; not an undefined/inconsistent state.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-016</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Stage 6</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Query against zero ingested content</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>A business with no successfully ingested pages</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>A business whose scrape entirely failed</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Run a RAG query against it.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Returns an empty/honest no-evidence result, not a crash or a hallucinated answer.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-017</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Stage 7</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Maps API quota/error handling</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Google Maps API key exhausted or erroring</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>A run where the Maps API returns errors for every call</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Run the pipeline through the Maps stage under this condition.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Pipeline degrades gracefully (Maps-derived fields left empty/unknown) rather than crashing or fabricating Maps data -- same class of guarantee already proven for Serper.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-018</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Stage 7</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Duplicate/multiple Maps listings</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A business has multiple branch listings</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>A chain with several Maps entries under similar names</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Run Maps matching against the target business.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>The correct listing is matched (or ambiguity is flagged) rather than an arbitrary/wrong branch being silently attached.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-019</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Stage 8</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Accuracy Check</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Fully empty business record</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>A business record with no populated fields at all</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>A record where every extractable field failed</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Run the accuracy/DataState scoring over it.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Resolves to the correct lowest DataState value and a clear low/zero score -- no crash, no exception.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-020</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Concurrent writes</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Two pipeline runs write the same domain concurrently</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Run storage layer</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Two parallel runs both discover the same business domain</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Trigger concurrent writes to the same domain's storage folder.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>No corrupted/partially-written files; writes are safely serialized or isolated (staging/commit pattern holds under concurrency).</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-021</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Corrupted index recovery</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>crawl_index.csv is malformed on load</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Run storage layer</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>A hand-corrupted/truncated crawl_index.csv</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Start the pipeline with this file present.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Pipeline either recovers gracefully (skips bad rows) or fails with a clear error -- never a silent, partial, or crashing load.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-022</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>REST/API</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Malformed request body</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Genuinely broken JSON, not a business-validation error</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>POST to /api/v1/pipeline/run</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>A request body that is not valid JSON at all</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Send the malformed request.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Returns 422 with a clear parse error, never a 500 or an unhandled exception.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-023</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>REST/API</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Job cancellation promptness</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Cancel a job mid-flight during expensive work (e.g. mid-crawl)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Submit a job, then cancel while it's actively scraping</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>A long-running job</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Cancel and measure how quickly in-flight work actually stops (not just the status flag flipping).</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>In-flight work (HTTP fetches, LLM calls) is actually aborted promptly, not left running to completion in the background after cancellation is acknowledged.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-024</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>REST/API</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Idempotency record lifecycle</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Idempotency-Key store growth over time</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Submit many distinct Idempotency-Keys over time</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Repeated distinct requests</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Inspect whether idempotency records are ever expired/evicted.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Records either expire after a reasonable window or the growth is a documented, bounded, accepted tradeoff -- not unbounded memory growth.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GAP-FUNC-025</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>REST/API</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Cursor pagination edge cases</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Invalid or past-the-end cursor value</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Call a paginated listing endpoint</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>cursor=&lt;garbage&gt; and cursor=&lt;value past the last page&gt;</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Call the endpoint with both.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Returns a clear 400/empty-page response, never a crash or an out-of-range exception.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GAP-PERF-005</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Memory over a large run</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Many businesses processed in one job</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Run a job targeting a large result_limit</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>A job processing dozens of businesses in one run</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Monitor process memory across the full run.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Memory stays bounded/does not grow unboundedly (no leak) across a long run.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>GAP-PERF-006</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sustained high job-submission rate</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>20-50 jobs submitted in quick succession</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Submit far more concurrent jobs than the PERF-001 baseline (5)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>A burst of 20-50 simultaneous job submissions</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Submit the burst and observe where responsiveness/isolation first degrades.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>The service degrades predictably (queues, or a documented concurrency ceiling) rather than becoming unresponsive or corrupting job state.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>